<commit_message>
Added printing of the dataframes on the web page
</commit_message>
<xml_diff>
--- a/tax_report.xlsx
+++ b/tax_report.xlsx
@@ -976,6 +976,39 @@
       </c>
     </row>
     <row r="7" spans="1:16" s="6" customFormat="1">
+      <c r="A7" s="6">
+        <v>0</v>
+      </c>
+      <c r="B7" s="6">
+        <v>0</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6">
+        <v>0</v>
+      </c>
+      <c r="G7" s="6">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
+        <v>0</v>
+      </c>
       <c r="L7" s="6">
         <v>93190.32000000001</v>
       </c>

</xml_diff>

<commit_message>
Updated the comments for 2025 tax form. Modified the cell comments formatting.
</commit_message>
<xml_diff>
--- a/tax_report.xlsx
+++ b/tax_report.xlsx
@@ -89,12 +89,21 @@
       <text>
         <r>
           <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Into Pit38 C.22</t>
+            <sz val="11"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Into PIT-38 -&gt; Income -&gt; 
+Other revenue, including revenue earned abroad and revenue from sale of virtual currencies - Article 30B(1A) of the Act -&gt;
+Revenue (zł) - PIT-38 C22
+Also:
+Tick "Revenue earned abroad";
+Income earned abroad -&gt;
+Income type - other revenue, including revenue earned abroad -&gt;
+Income earned abroad (zł) - PIT-ZG C29
+and 0zł into:
+Show tax on this income paid abroad (zł) - PIT-ZG C30                    </t>
         </r>
       </text>
     </comment>
@@ -102,12 +111,14 @@
       <text>
         <r>
           <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Into Pit38 C.23</t>
+            <sz val="11"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Into PIT-38 -&gt; Income -&gt;
+Other revenue, including revenue earned abroad and revenue from sale of virtual currencies - Article 30B(1A) of the Act -&gt;
+Tax deductible expenses (zł) - PIT-38 C.23                    </t>
         </r>
       </text>
     </comment>
@@ -143,11 +154,24 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
+          <t>= Income PLN * 0.19</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
           <t>= TaxWitholded USD * DividendUSDRate D-1 PLN</t>
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -156,19 +180,6 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>= Income PLN * 0.19</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
           <t>= sum(TaxPL PLN) - sum(TaxWitholdedInUS PLN)</t>
         </r>
       </text>
@@ -177,12 +188,15 @@
       <text>
         <r>
           <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Into Pit38 G.46</t>
+            <sz val="11"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Into PIT-38 -&gt; Income -&gt;
+Other revenue, including revenue earned abroad and revenue from sale of virtual currencies - Article 30B(1A) of the Act -&gt;
+Lump-sum tax on revenue (income) earned abroad -&gt;
+Lump-sum tax (zł) - PIT-38 G.47                    </t>
         </r>
       </text>
     </comment>
@@ -190,12 +204,15 @@
       <text>
         <r>
           <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Into Pit38 G.45</t>
+            <sz val="11"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Into PIT-38 -&gt; Income -&gt;
+Other revenue, including revenue earned abroad and revenue from sale of virtual currencies - Article 30B(1A) of the Act -&gt;
+Lump-sum tax on revenue (income) earned abroad -&gt;
+Tax paid abroad (zł) - PIT-38 G.48                    </t>
         </r>
       </text>
     </comment>
@@ -278,10 +295,10 @@
     <t>Income PLN</t>
   </si>
   <si>
+    <t>TaxPL PLN</t>
+  </si>
+  <si>
     <t>TaxWitholdedInUS PLN</t>
-  </si>
-  <si>
-    <t>TaxPL PLN</t>
   </si>
   <si>
     <t>TaxDue PLN</t>
@@ -976,39 +993,6 @@
       </c>
     </row>
     <row r="7" spans="1:16" s="6" customFormat="1">
-      <c r="A7" s="6">
-        <v>0</v>
-      </c>
-      <c r="B7" s="6">
-        <v>0</v>
-      </c>
-      <c r="C7" s="6">
-        <v>0</v>
-      </c>
-      <c r="D7" s="6">
-        <v>0</v>
-      </c>
-      <c r="E7" s="6">
-        <v>0</v>
-      </c>
-      <c r="F7" s="6">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6">
-        <v>0</v>
-      </c>
-      <c r="H7" s="6">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6">
-        <v>0</v>
-      </c>
-      <c r="K7" s="6">
-        <v>0</v>
-      </c>
       <c r="L7" s="6">
         <v>93190.32000000001</v>
       </c>
@@ -1041,8 +1025,8 @@
     <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1089,10 +1073,10 @@
         <v>1750.75</v>
       </c>
       <c r="F2" s="2">
+        <v>332.64</v>
+      </c>
+      <c r="G2" s="2">
         <v>262.61</v>
-      </c>
-      <c r="G2" s="2">
-        <v>332.64</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="6" customFormat="1">
@@ -1100,10 +1084,10 @@
         <v>1750.75</v>
       </c>
       <c r="F3" s="6">
+        <v>332.64</v>
+      </c>
+      <c r="G3" s="6">
         <v>262.61</v>
-      </c>
-      <c r="G3" s="6">
-        <v>332.64</v>
       </c>
       <c r="H3" s="6">
         <v>70.03</v>

</xml_diff>